<commit_message>
maakt gebruik van scans-map
</commit_message>
<xml_diff>
--- a/input/Documentenlijst.xlsx
+++ b/input/Documentenlijst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronaldkoenis/eclipse-workspace/maakmdto/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F569B03C-BEF7-CF48-951D-8202B6A31D38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA95F4B-19B9-7C47-B823-52980BEA6FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-6940" yWindow="-27480" windowWidth="39100" windowHeight="17960" xr2:uid="{CD58AC6D-95E4-3D46-BF36-5AD7BB9721C7}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="366" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="189">
   <si>
     <t>agendapunt</t>
   </si>
@@ -533,12 +533,6 @@
     <t>Vergaderdatum</t>
   </si>
   <si>
-    <t>2017-11-07/Programmabegroting 2018</t>
-  </si>
-  <si>
-    <t>2017-11-07</t>
-  </si>
-  <si>
     <t>A1 - Amendement Streekbelangen, LL, PvdA + HVV - Verlaging tarieven binnensport - aangenomen - r 20171107.pdf</t>
   </si>
   <si>
@@ -572,9 +566,6 @@
     <t>deze niet.txt</t>
   </si>
   <si>
-    <t>2018-03-06/alles</t>
-  </si>
-  <si>
     <t>Agenda Gemeenteraad_07-11-2017.pdf</t>
   </si>
   <si>
@@ -605,19 +596,10 @@
     <t>Programmabegroting 2018 (Def. na raad 20171107 - incl. A1 + A3).pdf</t>
   </si>
   <si>
-    <t>Agenda (gewijzigd) Gemeenteraad_06-03-2018 (20180301).pdf</t>
-  </si>
-  <si>
-    <t>2018-03-06</t>
-  </si>
-  <si>
-    <t>Besluitenlijst-BESL-INT_C257092D8760438382D756BBAAFB7F82 februari.pdf</t>
-  </si>
-  <si>
-    <t>Besluitenlijst-BESL-INT_3346CC83C70245C7A759CEC53465DD8F januari.pdf</t>
-  </si>
-  <si>
     <t>Bewerking</t>
+  </si>
+  <si>
+    <t>Scans</t>
   </si>
 </sst>
 </file>
@@ -1121,7 +1103,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1136,10 +1118,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="33" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="33" borderId="0" xfId="0" quotePrefix="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1541,7 +1521,7 @@
         <v>2</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>164</v>
@@ -1563,11 +1543,11 @@
       <c r="D2" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="G2" s="10" t="s">
-        <v>180</v>
+      <c r="F2" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G2" s="9" t="s">
+        <v>178</v>
       </c>
     </row>
     <row r="3" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1583,11 +1563,11 @@
       <c r="D3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F3" s="8" t="s">
-        <v>167</v>
-      </c>
-      <c r="G3" s="10" t="s">
-        <v>181</v>
+      <c r="F3" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>177</v>
       </c>
     </row>
     <row r="4" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1604,10 +1584,10 @@
         <v>10</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>177</v>
+        <v>188</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>175</v>
       </c>
     </row>
     <row r="5" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1624,10 +1604,10 @@
         <v>18</v>
       </c>
       <c r="F5" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G5" s="8" t="s">
         <v>166</v>
-      </c>
-      <c r="G5" s="9" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="6" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1644,10 +1624,10 @@
         <v>19</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>166</v>
+        <v>188</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
     </row>
     <row r="7" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1664,10 +1644,10 @@
         <v>20</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G7" s="9" t="s">
-        <v>170</v>
+        <v>188</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="8" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1684,10 +1664,10 @@
         <v>11</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>182</v>
+        <v>188</v>
+      </c>
+      <c r="G8" s="9" t="s">
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1704,10 +1684,10 @@
         <v>14</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>183</v>
+        <v>188</v>
+      </c>
+      <c r="G9" s="9" t="s">
+        <v>180</v>
       </c>
     </row>
     <row r="10" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1724,10 +1704,10 @@
         <v>12</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>184</v>
+        <v>188</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>181</v>
       </c>
     </row>
     <row r="11" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1744,10 +1724,10 @@
         <v>13</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>185</v>
+        <v>188</v>
+      </c>
+      <c r="G11" s="9" t="s">
+        <v>182</v>
       </c>
     </row>
     <row r="12" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1764,10 +1744,10 @@
         <v>15</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>186</v>
+        <v>188</v>
+      </c>
+      <c r="G12" s="9" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1784,10 +1764,10 @@
         <v>16</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>187</v>
+        <v>188</v>
+      </c>
+      <c r="G13" s="9" t="s">
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1804,10 +1784,10 @@
         <v>21</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>171</v>
+        <v>188</v>
+      </c>
+      <c r="G14" s="8" t="s">
+        <v>169</v>
       </c>
     </row>
     <row r="15" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1824,10 +1804,10 @@
         <v>22</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G15" s="9" t="s">
-        <v>172</v>
+        <v>188</v>
+      </c>
+      <c r="G15" s="8" t="s">
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1844,10 +1824,10 @@
         <v>23</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G16" s="9" t="s">
-        <v>173</v>
+        <v>188</v>
+      </c>
+      <c r="G16" s="8" t="s">
+        <v>171</v>
       </c>
     </row>
     <row r="17" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1864,10 +1844,10 @@
         <v>24</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G17" s="9" t="s">
-        <v>174</v>
+        <v>188</v>
+      </c>
+      <c r="G17" s="8" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="18" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1884,10 +1864,10 @@
         <v>25</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>166</v>
+        <v>188</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="19" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1904,10 +1884,10 @@
         <v>26</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>166</v>
+        <v>188</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="20" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1924,10 +1904,10 @@
         <v>8</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G20" s="10" t="s">
-        <v>188</v>
+        <v>188</v>
+      </c>
+      <c r="G20" s="9" t="s">
+        <v>185</v>
       </c>
     </row>
     <row r="21" spans="1:7" s="4" customFormat="1" x14ac:dyDescent="0.2">
@@ -1944,10 +1924,10 @@
         <v>9</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>166</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>189</v>
+        <v>188</v>
+      </c>
+      <c r="G21" s="9" t="s">
+        <v>186</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.2">
@@ -1963,7 +1943,13 @@
       <c r="D22" t="s">
         <v>27</v>
       </c>
-      <c r="F22" s="11"/>
+      <c r="F22" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G22" t="str">
+        <f t="shared" ref="G22:G26" si="0">C22&amp;".pdf"</f>
+        <v>6228528.pdf</v>
+      </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
@@ -1978,11 +1964,12 @@
       <c r="D23" t="s">
         <v>28</v>
       </c>
-      <c r="F23" s="11" t="s">
-        <v>191</v>
-      </c>
-      <c r="G23" s="10" t="s">
-        <v>190</v>
+      <c r="F23" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G23" t="str">
+        <f t="shared" si="0"/>
+        <v>6243883.pdf</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.2">
@@ -1998,11 +1985,12 @@
       <c r="D24" t="s">
         <v>30</v>
       </c>
-      <c r="F24" s="11" t="s">
-        <v>191</v>
-      </c>
-      <c r="G24" s="10" t="s">
-        <v>193</v>
+      <c r="F24" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G24" t="str">
+        <f t="shared" si="0"/>
+        <v>6194939.pdf</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -2033,11 +2021,12 @@
       <c r="D26" t="s">
         <v>32</v>
       </c>
-      <c r="F26" s="11" t="s">
-        <v>191</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>192</v>
+      <c r="F26" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G26" t="str">
+        <f t="shared" si="0"/>
+        <v>6194952.pdf</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -2054,7 +2043,7 @@
         <v>34</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G27" t="str">
         <f>C27&amp;".pdf"</f>
@@ -2075,7 +2064,7 @@
         <v>35</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G28" t="str">
         <f>C28&amp;".pdf"</f>
@@ -2097,7 +2086,7 @@
       </c>
       <c r="F29" s="4"/>
       <c r="G29" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.2">
@@ -2114,10 +2103,10 @@
         <v>37</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G30" t="str">
-        <f>C30&amp;".pdf"</f>
+        <f t="shared" ref="G30:G61" si="1">C30&amp;".pdf"</f>
         <v>6269707.pdf</v>
       </c>
     </row>
@@ -2135,10 +2124,10 @@
         <v>38</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G31" t="str">
-        <f>C31&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6194987.pdf</v>
       </c>
     </row>
@@ -2156,10 +2145,10 @@
         <v>39</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G32" t="str">
-        <f>C32&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195019.pdf</v>
       </c>
     </row>
@@ -2177,10 +2166,10 @@
         <v>40</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G33" t="str">
-        <f>C33&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6194981.pdf</v>
       </c>
     </row>
@@ -2198,10 +2187,10 @@
         <v>41</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G34" t="str">
-        <f>C34&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6194982.pdf</v>
       </c>
     </row>
@@ -2219,10 +2208,10 @@
         <v>42</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G35" t="str">
-        <f>C35&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6194983.pdf</v>
       </c>
     </row>
@@ -2240,10 +2229,10 @@
         <v>43</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G36" t="str">
-        <f>C36&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6194984.pdf</v>
       </c>
     </row>
@@ -2261,10 +2250,10 @@
         <v>44</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G37" t="str">
-        <f>C37&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6194985.pdf</v>
       </c>
     </row>
@@ -2282,10 +2271,10 @@
         <v>45</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G38" t="str">
-        <f>C38&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6194988.pdf</v>
       </c>
     </row>
@@ -2303,10 +2292,10 @@
         <v>46</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G39" t="str">
-        <f>C39&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6269744.pdf</v>
       </c>
     </row>
@@ -2324,10 +2313,10 @@
         <v>47</v>
       </c>
       <c r="F40" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G40" t="str">
-        <f>C40&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6229927.pdf</v>
       </c>
     </row>
@@ -2345,10 +2334,10 @@
         <v>48</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G41" t="str">
-        <f>C41&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6229928.pdf</v>
       </c>
     </row>
@@ -2366,10 +2355,10 @@
         <v>49</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G42" t="str">
-        <f>C42&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195010.pdf</v>
       </c>
     </row>
@@ -2387,10 +2376,10 @@
         <v>50</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G43" t="str">
-        <f>C43&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195021.pdf</v>
       </c>
     </row>
@@ -2408,10 +2397,10 @@
         <v>51</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G44" t="str">
-        <f>C44&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195011.pdf</v>
       </c>
     </row>
@@ -2429,10 +2418,10 @@
         <v>52</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G45" t="str">
-        <f>C45&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195012.pdf</v>
       </c>
     </row>
@@ -2450,10 +2439,10 @@
         <v>53</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G46" t="str">
-        <f>C46&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195013.pdf</v>
       </c>
     </row>
@@ -2471,10 +2460,10 @@
         <v>54</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G47" t="str">
-        <f>C47&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195014.pdf</v>
       </c>
     </row>
@@ -2492,10 +2481,10 @@
         <v>55</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G48" t="str">
-        <f>C48&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195015.pdf</v>
       </c>
     </row>
@@ -2513,10 +2502,10 @@
         <v>56</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G49" t="str">
-        <f>C49&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195016.pdf</v>
       </c>
     </row>
@@ -2534,10 +2523,10 @@
         <v>57</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G50" t="str">
-        <f>C50&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195017.pdf</v>
       </c>
     </row>
@@ -2555,10 +2544,10 @@
         <v>58</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G51" t="str">
-        <f>C51&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195018.pdf</v>
       </c>
     </row>
@@ -2576,10 +2565,10 @@
         <v>59</v>
       </c>
       <c r="F52" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G52" t="str">
-        <f>C52&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6231660.pdf</v>
       </c>
     </row>
@@ -2597,10 +2586,10 @@
         <v>60</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G53" t="str">
-        <f>C53&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6235284.pdf</v>
       </c>
     </row>
@@ -2618,10 +2607,10 @@
         <v>61</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G54" t="str">
-        <f>C54&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6266837.pdf</v>
       </c>
     </row>
@@ -2639,10 +2628,10 @@
         <v>62</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G55" t="str">
-        <f>C55&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195047.pdf</v>
       </c>
     </row>
@@ -2660,10 +2649,10 @@
         <v>63</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G56" t="str">
-        <f>C56&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195044.pdf</v>
       </c>
     </row>
@@ -2681,10 +2670,10 @@
         <v>64</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G57" t="str">
-        <f>C57&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195043.pdf</v>
       </c>
     </row>
@@ -2702,10 +2691,10 @@
         <v>65</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G58" t="str">
-        <f>C58&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6231889.pdf</v>
       </c>
     </row>
@@ -2723,10 +2712,10 @@
         <v>66</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G59" t="str">
-        <f>C59&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195046.pdf</v>
       </c>
     </row>
@@ -2744,10 +2733,10 @@
         <v>67</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G60" t="str">
-        <f>C60&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6195045.pdf</v>
       </c>
     </row>
@@ -2765,10 +2754,10 @@
         <v>68</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G61" t="str">
-        <f>C61&amp;".pdf"</f>
+        <f t="shared" si="1"/>
         <v>6231890.pdf</v>
       </c>
     </row>
@@ -2786,10 +2775,10 @@
         <v>69</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G62" t="str">
-        <f>C62&amp;".pdf"</f>
+        <f t="shared" ref="G62:G86" si="2">C62&amp;".pdf"</f>
         <v>6195049.pdf</v>
       </c>
     </row>
@@ -2807,10 +2796,10 @@
         <v>70</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G63" t="str">
-        <f>C63&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195048.pdf</v>
       </c>
     </row>
@@ -2828,10 +2817,10 @@
         <v>71</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G64" t="str">
-        <f>C64&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195051.pdf</v>
       </c>
     </row>
@@ -2849,10 +2838,10 @@
         <v>72</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G65" t="str">
-        <f>C65&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195050.pdf</v>
       </c>
     </row>
@@ -2870,10 +2859,10 @@
         <v>73</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G66" t="str">
-        <f>C66&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195040.pdf</v>
       </c>
     </row>
@@ -2891,10 +2880,10 @@
         <v>74</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G67" t="str">
-        <f>C67&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195041.pdf</v>
       </c>
     </row>
@@ -2912,10 +2901,10 @@
         <v>75</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G68" t="str">
-        <f>C68&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195042.pdf</v>
       </c>
     </row>
@@ -2933,10 +2922,10 @@
         <v>76</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G69" t="str">
-        <f>C69&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195055.pdf</v>
       </c>
     </row>
@@ -2954,10 +2943,10 @@
         <v>77</v>
       </c>
       <c r="F70" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G70" t="str">
-        <f>C70&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195054.pdf</v>
       </c>
     </row>
@@ -2975,10 +2964,10 @@
         <v>78</v>
       </c>
       <c r="F71" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G71" t="str">
-        <f>C71&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195052.pdf</v>
       </c>
     </row>
@@ -2996,10 +2985,10 @@
         <v>79</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G72" t="str">
-        <f>C72&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195056.pdf</v>
       </c>
     </row>
@@ -3017,10 +3006,10 @@
         <v>80</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G73" t="str">
-        <f>C73&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195053.pdf</v>
       </c>
     </row>
@@ -3038,10 +3027,10 @@
         <v>81</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G74" t="str">
-        <f>C74&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6269924.pdf</v>
       </c>
     </row>
@@ -3059,10 +3048,10 @@
         <v>82</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G75" t="str">
-        <f>C75&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195081.pdf</v>
       </c>
     </row>
@@ -3080,10 +3069,10 @@
         <v>83</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G76" t="str">
-        <f>C76&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195079.pdf</v>
       </c>
     </row>
@@ -3101,10 +3090,10 @@
         <v>84</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G77" t="str">
-        <f>C77&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195078.pdf</v>
       </c>
     </row>
@@ -3122,10 +3111,10 @@
         <v>85</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G78" t="str">
-        <f>C78&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195080.pdf</v>
       </c>
     </row>
@@ -3143,10 +3132,10 @@
         <v>86</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G79" t="str">
-        <f>C79&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195076.pdf</v>
       </c>
     </row>
@@ -3164,10 +3153,10 @@
         <v>87</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G80" t="str">
-        <f>C80&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195082.pdf</v>
       </c>
     </row>
@@ -3185,10 +3174,10 @@
         <v>88</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G81" t="str">
-        <f>C81&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195077.pdf</v>
       </c>
     </row>
@@ -3206,10 +3195,10 @@
         <v>89</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G82" t="str">
-        <f>C82&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195083.pdf</v>
       </c>
     </row>
@@ -3227,10 +3216,10 @@
         <v>90</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G83" t="str">
-        <f>C83&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195085.pdf</v>
       </c>
     </row>
@@ -3248,10 +3237,10 @@
         <v>91</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G84" t="str">
-        <f>C84&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195087.pdf</v>
       </c>
     </row>
@@ -3269,10 +3258,10 @@
         <v>92</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G85" t="str">
-        <f>C85&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195086.pdf</v>
       </c>
     </row>
@@ -3290,10 +3279,10 @@
         <v>93</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G86" t="str">
-        <f>C86&amp;".pdf"</f>
+        <f t="shared" si="2"/>
         <v>6195084.pdf</v>
       </c>
     </row>
@@ -3311,10 +3300,10 @@
         <v>94</v>
       </c>
       <c r="F87" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G87" t="str">
-        <f t="shared" ref="G87:G150" si="0">C87&amp;".pdf"</f>
+        <f t="shared" ref="G87:G150" si="3">C87&amp;".pdf"</f>
         <v>6269977.pdf</v>
       </c>
     </row>
@@ -3332,10 +3321,10 @@
         <v>95</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G88" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195109.pdf</v>
       </c>
     </row>
@@ -3353,10 +3342,10 @@
         <v>96</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G89" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195110.pdf</v>
       </c>
     </row>
@@ -3374,10 +3363,10 @@
         <v>97</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G90" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195111.pdf</v>
       </c>
     </row>
@@ -3395,10 +3384,10 @@
         <v>98</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G91" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6270017.pdf</v>
       </c>
     </row>
@@ -3416,10 +3405,10 @@
         <v>99</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G92" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195115.pdf</v>
       </c>
     </row>
@@ -3437,10 +3426,10 @@
         <v>100</v>
       </c>
       <c r="F93" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G93" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6238018.pdf</v>
       </c>
     </row>
@@ -3458,10 +3447,10 @@
         <v>101</v>
       </c>
       <c r="F94" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G94" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195116.pdf</v>
       </c>
     </row>
@@ -3479,10 +3468,10 @@
         <v>102</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G95" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6238017.pdf</v>
       </c>
     </row>
@@ -3500,10 +3489,10 @@
         <v>103</v>
       </c>
       <c r="F96" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G96" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195117.pdf</v>
       </c>
     </row>
@@ -3521,10 +3510,10 @@
         <v>104</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G97" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195118.pdf</v>
       </c>
     </row>
@@ -3542,10 +3531,10 @@
         <v>105</v>
       </c>
       <c r="F98" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G98" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6238016.pdf</v>
       </c>
     </row>
@@ -3563,10 +3552,10 @@
         <v>106</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G99" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6270073.pdf</v>
       </c>
     </row>
@@ -3584,10 +3573,10 @@
         <v>107</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G100" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195139.pdf</v>
       </c>
     </row>
@@ -3605,10 +3594,10 @@
         <v>108</v>
       </c>
       <c r="F101" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G101" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195140.pdf</v>
       </c>
     </row>
@@ -3626,10 +3615,10 @@
         <v>109</v>
       </c>
       <c r="F102" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G102" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195141.pdf</v>
       </c>
     </row>
@@ -3647,10 +3636,10 @@
         <v>110</v>
       </c>
       <c r="F103" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G103" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6270097.pdf</v>
       </c>
     </row>
@@ -3668,10 +3657,10 @@
         <v>111</v>
       </c>
       <c r="F104" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G104" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6227443.pdf</v>
       </c>
     </row>
@@ -3689,10 +3678,10 @@
         <v>112</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G105" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6227448.pdf</v>
       </c>
     </row>
@@ -3710,10 +3699,10 @@
         <v>113</v>
       </c>
       <c r="F106" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G106" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195166.pdf</v>
       </c>
     </row>
@@ -3731,10 +3720,10 @@
         <v>114</v>
       </c>
       <c r="F107" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G107" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195167.pdf</v>
       </c>
     </row>
@@ -3752,10 +3741,10 @@
         <v>115</v>
       </c>
       <c r="F108" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G108" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6270138.pdf</v>
       </c>
     </row>
@@ -3773,10 +3762,10 @@
         <v>116</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G109" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195241.pdf</v>
       </c>
     </row>
@@ -3794,10 +3783,10 @@
         <v>117</v>
       </c>
       <c r="F110" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G110" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195242.pdf</v>
       </c>
     </row>
@@ -3815,10 +3804,10 @@
         <v>118</v>
       </c>
       <c r="F111" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G111" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195240.pdf</v>
       </c>
     </row>
@@ -3836,10 +3825,10 @@
         <v>119</v>
       </c>
       <c r="F112" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G112" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195237.pdf</v>
       </c>
     </row>
@@ -3857,10 +3846,10 @@
         <v>120</v>
       </c>
       <c r="F113" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G113" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195239.pdf</v>
       </c>
     </row>
@@ -3878,10 +3867,10 @@
         <v>121</v>
       </c>
       <c r="F114" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G114" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195243.pdf</v>
       </c>
     </row>
@@ -3899,10 +3888,10 @@
         <v>122</v>
       </c>
       <c r="F115" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G115" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6270156.pdf</v>
       </c>
     </row>
@@ -3920,10 +3909,10 @@
         <v>123</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G116" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6227460.pdf</v>
       </c>
     </row>
@@ -3941,10 +3930,10 @@
         <v>124</v>
       </c>
       <c r="F117" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G117" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6227466.pdf</v>
       </c>
     </row>
@@ -3962,10 +3951,10 @@
         <v>125</v>
       </c>
       <c r="F118" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G118" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195251.pdf</v>
       </c>
     </row>
@@ -3983,10 +3972,10 @@
         <v>126</v>
       </c>
       <c r="F119" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G119" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195252.pdf</v>
       </c>
     </row>
@@ -4004,10 +3993,10 @@
         <v>127</v>
       </c>
       <c r="F120" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G120" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6270169.pdf</v>
       </c>
     </row>
@@ -4025,10 +4014,10 @@
         <v>128</v>
       </c>
       <c r="F121" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G121" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195277.pdf</v>
       </c>
     </row>
@@ -4046,10 +4035,10 @@
         <v>129</v>
       </c>
       <c r="F122" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G122" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195278.pdf</v>
       </c>
     </row>
@@ -4067,10 +4056,10 @@
         <v>130</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G123" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6270194.pdf</v>
       </c>
     </row>
@@ -4088,10 +4077,10 @@
         <v>131</v>
       </c>
       <c r="F124" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G124" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195386.pdf</v>
       </c>
     </row>
@@ -4109,10 +4098,10 @@
         <v>132</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G125" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195387.pdf</v>
       </c>
     </row>
@@ -4130,10 +4119,10 @@
         <v>133</v>
       </c>
       <c r="F126" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G126" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195388.pdf</v>
       </c>
     </row>
@@ -4151,10 +4140,10 @@
         <v>134</v>
       </c>
       <c r="F127" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G127" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195389.pdf</v>
       </c>
     </row>
@@ -4172,10 +4161,10 @@
         <v>135</v>
       </c>
       <c r="F128" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G128" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195390.pdf</v>
       </c>
     </row>
@@ -4193,10 +4182,10 @@
         <v>136</v>
       </c>
       <c r="F129" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G129" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6270258.pdf</v>
       </c>
     </row>
@@ -4214,10 +4203,10 @@
         <v>137</v>
       </c>
       <c r="F130" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G130" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195455.pdf</v>
       </c>
     </row>
@@ -4235,10 +4224,10 @@
         <v>138</v>
       </c>
       <c r="F131" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G131" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195451.pdf</v>
       </c>
     </row>
@@ -4256,10 +4245,10 @@
         <v>139</v>
       </c>
       <c r="F132" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G132" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195452.pdf</v>
       </c>
     </row>
@@ -4277,10 +4266,10 @@
         <v>140</v>
       </c>
       <c r="F133" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G133" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195454.pdf</v>
       </c>
     </row>
@@ -4298,10 +4287,10 @@
         <v>142</v>
       </c>
       <c r="F134" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G134" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6271546.pdf</v>
       </c>
     </row>
@@ -4319,10 +4308,10 @@
         <v>143</v>
       </c>
       <c r="F135" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G135" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6216877.pdf</v>
       </c>
     </row>
@@ -4340,10 +4329,10 @@
         <v>144</v>
       </c>
       <c r="F136" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G136" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6216881.pdf</v>
       </c>
     </row>
@@ -4361,10 +4350,10 @@
         <v>145</v>
       </c>
       <c r="F137" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G137" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6216883.pdf</v>
       </c>
     </row>
@@ -4382,10 +4371,10 @@
         <v>146</v>
       </c>
       <c r="F138" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G138" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6270307.pdf</v>
       </c>
     </row>
@@ -4403,10 +4392,10 @@
         <v>147</v>
       </c>
       <c r="F139" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G139" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6217332.pdf</v>
       </c>
     </row>
@@ -4424,10 +4413,10 @@
         <v>148</v>
       </c>
       <c r="F140" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G140" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195470.pdf</v>
       </c>
     </row>
@@ -4445,10 +4434,10 @@
         <v>149</v>
       </c>
       <c r="F141" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G141" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195473.pdf</v>
       </c>
     </row>
@@ -4466,10 +4455,10 @@
         <v>150</v>
       </c>
       <c r="F142" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G142" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195468.pdf</v>
       </c>
     </row>
@@ -4487,10 +4476,10 @@
         <v>151</v>
       </c>
       <c r="F143" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G143" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6252419.pdf</v>
       </c>
     </row>
@@ -4508,10 +4497,10 @@
         <v>152</v>
       </c>
       <c r="F144" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G144" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6252420.pdf</v>
       </c>
     </row>
@@ -4529,10 +4518,10 @@
         <v>153</v>
       </c>
       <c r="F145" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G145" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6256604.pdf</v>
       </c>
     </row>
@@ -4550,10 +4539,10 @@
         <v>154</v>
       </c>
       <c r="F146" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G146" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6201992.pdf</v>
       </c>
     </row>
@@ -4571,10 +4560,10 @@
         <v>155</v>
       </c>
       <c r="F147" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G147" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6228529.pdf</v>
       </c>
     </row>
@@ -4592,10 +4581,10 @@
         <v>156</v>
       </c>
       <c r="F148" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G148" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6228530.pdf</v>
       </c>
     </row>
@@ -4613,10 +4602,10 @@
         <v>157</v>
       </c>
       <c r="F149" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G149" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6228531.pdf</v>
       </c>
     </row>
@@ -4634,10 +4623,10 @@
         <v>158</v>
       </c>
       <c r="F150" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G150" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="3"/>
         <v>6195501.pdf</v>
       </c>
     </row>
@@ -4655,10 +4644,10 @@
         <v>159</v>
       </c>
       <c r="F151" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G151" t="str">
-        <f t="shared" ref="G151:G154" si="1">C151&amp;".pdf"</f>
+        <f t="shared" ref="G151:G154" si="4">C151&amp;".pdf"</f>
         <v>6243879.pdf</v>
       </c>
     </row>
@@ -4676,10 +4665,10 @@
         <v>160</v>
       </c>
       <c r="F152" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G152" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>6243880.pdf</v>
       </c>
     </row>
@@ -4697,10 +4686,10 @@
         <v>161</v>
       </c>
       <c r="F153" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G153" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>6256571.pdf</v>
       </c>
     </row>
@@ -4718,10 +4707,10 @@
         <v>162</v>
       </c>
       <c r="F154" s="4" t="s">
-        <v>179</v>
+        <v>188</v>
       </c>
       <c r="G154" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
         <v>6256121.pdf</v>
       </c>
     </row>

</xml_diff>

<commit_message>
met trucje om downloads van mp4 te voorkomen
</commit_message>
<xml_diff>
--- a/input/Documentenlijst.xlsx
+++ b/input/Documentenlijst.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ronaldkoenis/eclipse-workspace/maakmdto/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EA95F4B-19B9-7C47-B823-52980BEA6FE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{073D5796-9CD0-AA49-A8B6-E7B4A2458FD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-6940" yWindow="-27480" windowWidth="39100" windowHeight="17960" xr2:uid="{CD58AC6D-95E4-3D46-BF36-5AD7BB9721C7}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="189">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="370" uniqueCount="193">
   <si>
     <t>agendapunt</t>
   </si>
@@ -600,6 +600,18 @@
   </si>
   <si>
     <t>Scans</t>
+  </si>
+  <si>
+    <t>Videotulen.mp4</t>
+  </si>
+  <si>
+    <t>375549-media-audio-1</t>
+  </si>
+  <si>
+    <t>466528-media-video-1</t>
+  </si>
+  <si>
+    <t>audiotulen.aac</t>
   </si>
 </sst>
 </file>
@@ -1103,7 +1115,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1120,6 +1132,9 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="6"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1495,7 +1510,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6DCD69E2-47BC-5E4E-B72B-254DA74E6572}">
-  <dimension ref="A1:G154"/>
+  <dimension ref="A1:G156"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="15.33203125" bestFit="1" customWidth="1"/>
@@ -4714,6 +4729,29 @@
         <v>6256121.pdf</v>
       </c>
     </row>
+    <row r="155" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A155" s="1"/>
+      <c r="C155" s="10" t="s">
+        <v>191</v>
+      </c>
+      <c r="F155" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G155" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="156" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C156" s="10" t="s">
+        <v>190</v>
+      </c>
+      <c r="F156" s="4" t="s">
+        <v>188</v>
+      </c>
+      <c r="G156" t="s">
+        <v>192</v>
+      </c>
+    </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:G21">
     <sortCondition ref="G4:G21"/>

</xml_diff>